<commit_message>
actualización ficha tecnica equipos
</commit_message>
<xml_diff>
--- a/Trimestre II/PROJECT.NAIAPP/Plantilla de Costos programadores.xlsx
+++ b/Trimestre II/PROJECT.NAIAPP/Plantilla de Costos programadores.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="120" uniqueCount="94">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="133" uniqueCount="105">
   <si>
     <t> Salario de programadores según experiencia en Colombia</t>
   </si>
@@ -236,25 +236,31 @@
     <t>Dirige el proyecto</t>
   </si>
   <si>
-    <t>tipo de pc</t>
-  </si>
-  <si>
-    <t>procesador</t>
-  </si>
-  <si>
-    <t>ram</t>
-  </si>
-  <si>
-    <t>almacenamiento</t>
-  </si>
-  <si>
-    <t>tarjeta de video</t>
-  </si>
-  <si>
-    <t>fuente</t>
-  </si>
-  <si>
-    <t>area</t>
+    <t>Tipo de equipo</t>
+  </si>
+  <si>
+    <t>Procesador</t>
+  </si>
+  <si>
+    <t>RAM</t>
+  </si>
+  <si>
+    <t>Almacenamiento</t>
+  </si>
+  <si>
+    <t>Tarjeta de video</t>
+  </si>
+  <si>
+    <t>Fuente</t>
+  </si>
+  <si>
+    <t>ÁREA</t>
+  </si>
+  <si>
+    <t>Sistema operativo</t>
+  </si>
+  <si>
+    <t>Tipo de disco</t>
   </si>
   <si>
     <t>Portatil</t>
@@ -269,15 +275,18 @@
     <t>SSD 512 GB</t>
   </si>
   <si>
-    <t>n/a</t>
-  </si>
-  <si>
     <t>N/A</t>
   </si>
   <si>
     <t xml:space="preserve">desarrollador </t>
   </si>
   <si>
+    <t>Windows/Linux</t>
+  </si>
+  <si>
+    <t>ssd</t>
+  </si>
+  <si>
     <t>PC Servidor</t>
   </si>
   <si>
@@ -299,7 +308,31 @@
     <t>Servidores</t>
   </si>
   <si>
+    <t>Linux</t>
+  </si>
+  <si>
+    <t>hdd y ssd</t>
+  </si>
+  <si>
+    <t>AMD Ryzen 5</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 8 GB</t>
+  </si>
+  <si>
+    <t>512GB</t>
+  </si>
+  <si>
+    <t>Graficos integrados</t>
+  </si>
+  <si>
+    <t>N/a</t>
+  </si>
+  <si>
     <t>Administrativo</t>
+  </si>
+  <si>
+    <t>Windows 11</t>
   </si>
 </sst>
 </file>
@@ -314,7 +347,7 @@
     <numFmt numFmtId="168" formatCode="_-&quot;$&quot;\ * #,##0_-;\-&quot;$&quot;\ * #,##0_-;_-&quot;$&quot;\ * &quot;-&quot;?_-;_-@"/>
     <numFmt numFmtId="169" formatCode="_-&quot;$&quot;\ * #,##0.00_-;\-&quot;$&quot;\ * #,##0.00_-;_-&quot;$&quot;\ * &quot;-&quot;??_-;_-@"/>
   </numFmts>
-  <fonts count="9">
+  <fonts count="11">
     <font>
       <sz val="11.0"/>
       <color theme="1"/>
@@ -349,6 +382,17 @@
       <name val="Quattrocento Sans"/>
     </font>
     <font>
+      <b/>
+      <color theme="1"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11.0"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
       <color theme="1"/>
       <name val="Arial"/>
     </font>
@@ -581,7 +625,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="53">
+  <cellXfs count="55">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -705,10 +749,16 @@
     <xf borderId="9" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="9" fillId="0" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" vertical="center"/>
+    </xf>
+    <xf borderId="9" fillId="0" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
+    </xf>
+    <xf borderId="9" fillId="0" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="9" fillId="0" fontId="10" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
   </cellXfs>
@@ -2746,15 +2796,16 @@
   <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.0"/>
   <cols>
     <col customWidth="1" min="1" max="1" width="18.13"/>
-    <col customWidth="1" min="2" max="2" width="36.0"/>
-    <col customWidth="1" min="3" max="3" width="26.75"/>
-    <col customWidth="1" min="4" max="4" width="24.63"/>
-    <col customWidth="1" min="5" max="5" width="33.13"/>
-    <col customWidth="1" min="6" max="6" width="24.25"/>
-    <col customWidth="1" min="7" max="7" width="29.0"/>
+    <col customWidth="1" min="2" max="2" width="28.5"/>
+    <col customWidth="1" min="3" max="3" width="7.38"/>
+    <col customWidth="1" min="4" max="4" width="18.63"/>
+    <col customWidth="1" min="5" max="5" width="30.0"/>
+    <col customWidth="1" min="6" max="6" width="15.13"/>
+    <col customWidth="1" min="7" max="7" width="13.88"/>
+    <col customWidth="1" min="8" max="8" width="16.5"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="22.5" customHeight="1">
       <c r="A1" s="51" t="s">
         <v>72</v>
       </c>
@@ -2773,62 +2824,101 @@
       <c r="F1" s="51" t="s">
         <v>77</v>
       </c>
-      <c r="G1" s="51" t="s">
+      <c r="G1" s="52" t="s">
         <v>78</v>
       </c>
+      <c r="H1" s="52" t="s">
+        <v>79</v>
+      </c>
+      <c r="I1" s="51" t="s">
+        <v>80</v>
+      </c>
     </row>
     <row r="2">
-      <c r="A2" s="51" t="s">
-        <v>79</v>
-      </c>
-      <c r="B2" s="51" t="s">
-        <v>80</v>
-      </c>
-      <c r="C2" s="51" t="s">
+      <c r="A2" s="53" t="s">
         <v>81</v>
       </c>
-      <c r="D2" s="51" t="s">
+      <c r="B2" s="53" t="s">
         <v>82</v>
       </c>
-      <c r="E2" s="51" t="s">
+      <c r="C2" s="53" t="s">
         <v>83</v>
       </c>
-      <c r="F2" s="51" t="s">
+      <c r="D2" s="53" t="s">
         <v>84</v>
       </c>
-      <c r="G2" s="51" t="s">
+      <c r="E2" s="53" t="s">
         <v>85</v>
       </c>
+      <c r="F2" s="53" t="s">
+        <v>85</v>
+      </c>
+      <c r="G2" s="53" t="s">
+        <v>86</v>
+      </c>
+      <c r="H2" s="53" t="s">
+        <v>87</v>
+      </c>
+      <c r="I2" s="53" t="s">
+        <v>88</v>
+      </c>
     </row>
     <row r="3">
-      <c r="A3" s="51" t="s">
-        <v>86</v>
-      </c>
-      <c r="B3" s="52" t="s">
-        <v>87</v>
-      </c>
-      <c r="C3" s="51" t="s">
+      <c r="A3" s="53" t="s">
+        <v>89</v>
+      </c>
+      <c r="B3" s="54" t="s">
+        <v>90</v>
+      </c>
+      <c r="C3" s="53" t="s">
+        <v>91</v>
+      </c>
+      <c r="D3" s="53" t="s">
+        <v>92</v>
+      </c>
+      <c r="E3" s="54" t="s">
+        <v>93</v>
+      </c>
+      <c r="F3" s="54" t="s">
+        <v>94</v>
+      </c>
+      <c r="G3" s="53" t="s">
+        <v>95</v>
+      </c>
+      <c r="H3" s="53" t="s">
+        <v>96</v>
+      </c>
+      <c r="I3" s="53" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="53" t="s">
+        <v>81</v>
+      </c>
+      <c r="B4" s="54" t="s">
+        <v>98</v>
+      </c>
+      <c r="C4" s="53" t="s">
+        <v>99</v>
+      </c>
+      <c r="D4" s="53" t="s">
+        <v>100</v>
+      </c>
+      <c r="E4" s="53" t="s">
+        <v>101</v>
+      </c>
+      <c r="F4" s="53" t="s">
+        <v>102</v>
+      </c>
+      <c r="G4" s="54" t="s">
+        <v>103</v>
+      </c>
+      <c r="H4" s="53" t="s">
+        <v>104</v>
+      </c>
+      <c r="I4" s="53" t="s">
         <v>88</v>
-      </c>
-      <c r="D3" s="51" t="s">
-        <v>89</v>
-      </c>
-      <c r="E3" s="52" t="s">
-        <v>90</v>
-      </c>
-      <c r="F3" s="52" t="s">
-        <v>91</v>
-      </c>
-      <c r="G3" s="51" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="51" t="s">
-        <v>79</v>
-      </c>
-      <c r="G4" s="52" t="s">
-        <v>93</v>
       </c>
     </row>
   </sheetData>

</xml_diff>